<commit_message>
Add bags, stretcher, and refrigerator to the page
- Draft pocket layouts for the First-In bag, trauma bag, stretcher, and
  medicine refrigerator, drawn from the supply book photos
- Move the pediatric bag to the upper-right gap; heavy border for areas
  that aren't part of the wall (kind: bag)
- Optional pocket label and color fields in layout.json
- Rename refrigerator MED 1 to Cardiac Med
- Page shown at half size; status suffixes removed from area labels

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/truck_inventory.xlsx
+++ b/data/truck_inventory.xlsx
@@ -6362,7 +6362,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>MED 1</t>
+          <t>Cardiac Med</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>MED 1</t>
+          <t>Cardiac Med</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>MED 1</t>
+          <t>Cardiac Med</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>MED 1</t>
+          <t>Cardiac Med</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>MED 1</t>
+          <t>Cardiac Med</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>MED 1</t>
+          <t>Cardiac Med</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">

</xml_diff>